<commit_message>
Aggiornamento automatico P&C reports.xlsx
</commit_message>
<xml_diff>
--- a/P&C reports.xlsx
+++ b/P&C reports.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -817,12 +817,40 @@
           <t>Entrambe le serate</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>nero</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>wdamiata@gmail.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Entrambe le serate</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>